<commit_message>
Add email and phone verification with OTP, prevent duplicate registrations
</commit_message>
<xml_diff>
--- a/library-backend/users.xlsx
+++ b/library-backend/users.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -483,9 +483,23 @@
         <v>3/22/2026, 11:01:32 AM</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>OLALEYE IYANU JOHNSON</v>
+      </c>
+      <c r="B7" t="str">
+        <v>johnsonolaiyanu@gmail.com</v>
+      </c>
+      <c r="C7" t="str">
+        <v>08140227181</v>
+      </c>
+      <c r="D7" t="str">
+        <v>3/22/2026, 12:17:52 PM</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add structured user data display with HTML table format and improved JSON response
</commit_message>
<xml_diff>
--- a/library-backend/users.xlsx
+++ b/library-backend/users.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -497,9 +497,23 @@
         <v>3/22/2026, 12:17:52 PM</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>OLALEYE IYANU JOHNSON</v>
+      </c>
+      <c r="B8" t="str">
+        <v>johnsonolaiyanu@gmail.com</v>
+      </c>
+      <c r="C8" t="str">
+        <v>08140227181</v>
+      </c>
+      <c r="D8" t="str">
+        <v>3/22/2026, 12:39:40 PM</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add real-time duplicate email/phone validation endpoint for frontend
</commit_message>
<xml_diff>
--- a/library-backend/users.xlsx
+++ b/library-backend/users.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -511,9 +511,37 @@
         <v>3/22/2026, 12:39:40 PM</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>ibukun</v>
+      </c>
+      <c r="B9" t="str">
+        <v>johnsonolaiyanu@gmail.com</v>
+      </c>
+      <c r="C9" t="str">
+        <v>08140227181</v>
+      </c>
+      <c r="D9" t="str">
+        <v>3/22/2026, 12:54:19 PM</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>ibukun</v>
+      </c>
+      <c r="B10" t="str">
+        <v>johnsonolaiyanu@gmail.com</v>
+      </c>
+      <c r="C10" t="str">
+        <v>08140227181</v>
+      </c>
+      <c r="D10" t="str">
+        <v>3/22/2026, 12:55:52 PM</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update: user database with latest registrations
</commit_message>
<xml_diff>
--- a/library-backend/users.xlsx
+++ b/library-backend/users.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -539,9 +539,37 @@
         <v>3/22/2026, 12:55:52 PM</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>iyanu</v>
+      </c>
+      <c r="B11" t="str">
+        <v>johnsonolaiyanu@gmail.com</v>
+      </c>
+      <c r="C11" t="str">
+        <v>08140227181</v>
+      </c>
+      <c r="D11" t="str">
+        <v>3/22/2026, 1:04:32 PM</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>iyanu</v>
+      </c>
+      <c r="B12" t="str">
+        <v>johnsonolaiyanu@gmail.com</v>
+      </c>
+      <c r="C12" t="str">
+        <v>08140227181</v>
+      </c>
+      <c r="D12" t="str">
+        <v>3/22/2026, 1:21:44 PM</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>